<commit_message>
Fix Chinese bird names
</commit_message>
<xml_diff>
--- a/i18n/zh.xlsx
+++ b/i18n/zh.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Birds" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonuses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Birds" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bonuses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Goals" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Other" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Parameters" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -711,7 +711,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>阿尔塔米拉金莺</t>
+          <t>橙头拟鹂</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>亚马逊鹦鹉</t>
+          <t>亚马孙鹦哥</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>美国反嘴鹬</t>
+          <t>美洲反嘴鹬</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>美国悬崖燕子</t>
+          <t>红石燕</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>美国红隼</t>
+          <t>美洲隼</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>美洲斯特鹬</t>
+          <t>美洲蛎鹬</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>美国红尾鸲</t>
+          <t>橙尾鸲莺</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>安蒂奥基亚刷雀</t>
+          <t>安条基亚薮雀</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>灰喉鹟</t>
+          <t>灰喉蝇霸鹟</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>北极紫</t>
+          <t>北极海鹦</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚宜必思酒店</t>
+          <t>澳洲白鹮</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚苇莺</t>
+          <t>澳洲苇莺</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>州鸟</t>
+          <t>橙腹拟鹂</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>最大腹绿鹃</t>
+          <t>贝氏莺雀</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>黑颈鸊鷉</t>
+          <t>黑颈䴙䴘</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>澳洲身份证</t>
+          <t>澳洲鸢</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>黑头莺</t>
+          <t>白颊林莺</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>蓝色粗嘴雀</t>
+          <t>斑翅蓝彩鹀</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>蓝灰色捕蝇器</t>
+          <t>灰蓝蚋莺</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>蓝黄金刚牡马</t>
+          <t>蓝黄金刚鹦鹉</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>白腹雕</t>
+          <t>白腹隼雕</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>巴西凫</t>
+          <t>巴西鸭</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>古铜色牛鸟</t>
+          <t>铜色牛鹂</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>褐褐</t>
+          <t>褐鹈鹕</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>褐矢俏鸫</t>
+          <t>褐矢嘲鸫</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>虎皮栗马</t>
+          <t>虎皮鹦鹉</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>布什蒂特</t>
+          <t>丛山雀</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>珠颈斑禽</t>
+          <t>珠颈斑鹑</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>苇鹪鹩属</t>
+          <t>卡罗苇鹪鹩</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -6823,7 +6823,7 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>卡辛的麻雀</t>
+          <t>卡氏猛雀鹀</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
@@ -6915,7 +6915,7 @@
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>蓝莺</t>
+          <t>深蓝色林莺</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>烟彤雨燕</t>
+          <t>烟囱雨燕</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
@@ -7243,7 +7243,7 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>褐斑翅雀鵐</t>
+          <t>褐斑翅雀鹀</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
@@ -7471,7 +7471,7 @@
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>鸡尾牡马</t>
+          <t>鸡尾鹦鹉</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>叽叽柳莺</t>
+          <t>叽咋柳莺</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>普通小麻鳅</t>
+          <t>小苇鳽</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>扇尾沙锥</t>
+          <t>田鹬</t>
         </is>
       </c>
       <c r="F179" s="2" t="inlineStr">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>普通黄喉鸟</t>
+          <t>黄喉地莺</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>凤头奥彭多拉</t>
+          <t>冠拟椋鸟</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>涟林莺</t>
+          <t>波纹林莺</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>东罗塞拉</t>
+          <t>东澳玫瑰鹦鹉</t>
         </is>
       </c>
       <c r="F215" s="2" t="inlineStr">
@@ -10351,7 +10351,7 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>东部鞭鸟</t>
+          <t>绿鞭鸟</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>优雅的蜥蜴</t>
+          <t>优雅美洲咬鹃</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
@@ -11755,7 +11755,7 @@
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>红额金翅</t>
+          <t>红额金翅雀</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>欧金翅</t>
+          <t>欧金翅雀</t>
         </is>
       </c>
       <c r="F249" s="2" t="inlineStr">
@@ -12083,7 +12083,7 @@
       </c>
       <c r="E255" s="2" t="inlineStr">
         <is>
-          <t>欧洲粗暴</t>
+          <t>欧鸬鹚</t>
         </is>
       </c>
       <c r="F255" s="2" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="E256" s="2" t="inlineStr">
         <is>
-          <t>欧洲石聊</t>
+          <t>欧石䳭</t>
         </is>
       </c>
       <c r="F256" s="2" t="inlineStr">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t>纽西兰蕨</t>
+          <t>新西兰蝗莺</t>
         </is>
       </c>
       <c r="F259" s="2" t="inlineStr">
@@ -12395,7 +12395,7 @@
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>数额丝雀</t>
+          <t>金额丝雀</t>
         </is>
       </c>
       <c r="F262" s="2" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>粉红凤头栗马</t>
+          <t>粉红凤头鹦鹉</t>
         </is>
       </c>
       <c r="F268" s="2" t="inlineStr">
@@ -12747,7 +12747,7 @@
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>巨型鱼鸮</t>
+          <t>毛腿渔鸮</t>
         </is>
       </c>
       <c r="F270" s="2" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
-          <t>金头侏儒鸟</t>
+          <t>金头娇鹟</t>
         </is>
       </c>
       <c r="F275" s="2" t="inlineStr">
@@ -13167,7 +13167,7 @@
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>黄胸草鵐</t>
+          <t>黄胸草鹀</t>
         </is>
       </c>
       <c r="F279" s="2" t="inlineStr">
@@ -13207,7 +13207,7 @@
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
-          <t>草地蝇鵐</t>
+          <t>草地蝇鹀</t>
         </is>
       </c>
       <c r="F280" s="2" t="inlineStr">
@@ -13251,7 +13251,7 @@
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>灰猫喵鸫</t>
+          <t>灰猫嘲鸫</t>
         </is>
       </c>
       <c r="F281" s="2" t="inlineStr">
@@ -13479,7 +13479,7 @@
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>大凤头鹟</t>
+          <t>大冠蝇霸鹟</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
@@ -13523,7 +13523,7 @@
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>凤头鸊鷉</t>
+          <t>凤头䴙䴘</t>
         </is>
       </c>
       <c r="F287" s="2" t="inlineStr">
@@ -13831,7 +13831,7 @@
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>南亚鸨</t>
+          <t>印度鹭鸨</t>
         </is>
       </c>
       <c r="F294" s="2" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>伟大的波图</t>
+          <t>大林鸱</t>
         </is>
       </c>
       <c r="F296" s="2" t="inlineStr">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
-          <t>大斑点猕猴桃</t>
+          <t>大斑几维鸟</t>
         </is>
       </c>
       <c r="F297" s="2" t="inlineStr">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>走浣纱</t>
+          <t>走鹃</t>
         </is>
       </c>
       <c r="F306" s="2" t="inlineStr">
@@ -14651,7 +14651,7 @@
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>绿棉凫</t>
+          <t>绿棉鸭</t>
         </is>
       </c>
       <c r="F313" s="2" t="inlineStr">
@@ -14975,7 +14975,7 @@
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>雁灰</t>
+          <t>灰雁</t>
         </is>
       </c>
       <c r="F320" s="2" t="inlineStr">
@@ -15063,7 +15063,7 @@
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>海东青</t>
+          <t>矛隼</t>
         </is>
       </c>
       <c r="F322" s="2" t="inlineStr">
@@ -15403,7 +15403,7 @@
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>棕黄色 秋沙鸭</t>
+          <t>棕胁秋沙鸭</t>
         </is>
       </c>
       <c r="F330" s="2" t="inlineStr">
@@ -15443,7 +15443,7 @@
       </c>
       <c r="E331" s="2" t="inlineStr">
         <is>
-          <t>冠金翅</t>
+          <t>冠金翅雀</t>
         </is>
       </c>
       <c r="F331" s="2" t="inlineStr">
@@ -15607,7 +15607,7 @@
       </c>
       <c r="E335" s="2" t="inlineStr">
         <is>
-          <t>霍氏金葫芦</t>
+          <t>霍氏金鹃</t>
         </is>
       </c>
       <c r="F335" s="2" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="E346" s="2" t="inlineStr">
         <is>
-          <t>寿带印度</t>
+          <t>寿带鸟</t>
         </is>
       </c>
       <c r="F346" s="2" t="inlineStr">
@@ -16451,7 +16451,7 @@
       </c>
       <c r="E354" s="2" t="inlineStr">
         <is>
-          <t>啄羊驼</t>
+          <t>啄羊鹦鹉</t>
         </is>
       </c>
       <c r="F354" s="2" t="inlineStr">
@@ -16827,7 +16827,7 @@
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>鸮栗马</t>
+          <t>鸮鹦鹉</t>
         </is>
       </c>
       <c r="F363" s="2" t="inlineStr">
@@ -16999,7 +16999,7 @@
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>天青石彩旗</t>
+          <t>琉璃彩鹀</t>
         </is>
       </c>
       <c r="F367" s="2" t="inlineStr">
@@ -17047,7 +17047,7 @@
       </c>
       <c r="E368" s="2" t="inlineStr">
         <is>
-          <t>最少种子鹬</t>
+          <t>小籽鹬</t>
         </is>
       </c>
       <c r="F368" s="2" t="inlineStr">
@@ -17343,7 +17343,7 @@
       </c>
       <c r="E375" s="2" t="inlineStr">
         <is>
-          <t>林肯的麻雀</t>
+          <t>林氏带鹀</t>
         </is>
       </c>
       <c r="F375" s="2" t="inlineStr">
@@ -17599,7 +17599,7 @@
       </c>
       <c r="E381" s="2" t="inlineStr">
         <is>
-          <t>纵腹纹小鸮</t>
+          <t>纵纹腹小鸮</t>
         </is>
       </c>
       <c r="F381" s="2" t="inlineStr">
@@ -18043,7 +18043,7 @@
       </c>
       <c r="E391" s="2" t="inlineStr">
         <is>
-          <t>洋红色海燕</t>
+          <t>红紫圆尾鹱</t>
         </is>
       </c>
       <c r="F391" s="2" t="inlineStr">
@@ -18171,7 +18171,7 @@
       </c>
       <c r="E394" s="2" t="inlineStr">
         <is>
-          <t>米切氏凤头栗马</t>
+          <t>米切氏凤头鹦鹉</t>
         </is>
       </c>
       <c r="F394" s="2" t="inlineStr">
@@ -18351,7 +18351,7 @@
       </c>
       <c r="E398" s="2" t="inlineStr">
         <is>
-          <t>××林鸭</t>
+          <t>鬃林鸭</t>
         </is>
       </c>
       <c r="F398" s="2" t="inlineStr">
@@ -18479,7 +18479,7 @@
       </c>
       <c r="E401" s="2" t="inlineStr">
         <is>
-          <t>沼泽食籽虫</t>
+          <t>沼泽食籽雀</t>
         </is>
       </c>
       <c r="F401" s="2" t="inlineStr">
@@ -18703,7 +18703,7 @@
       </c>
       <c r="E406" s="2" t="inlineStr">
         <is>
-          <t>地中海海鸥</t>
+          <t>地中海鹱</t>
         </is>
       </c>
       <c r="F406" s="2" t="inlineStr">
@@ -18787,7 +18787,7 @@
       </c>
       <c r="E408" s="2" t="inlineStr">
         <is>
-          <t>密西西比风筝</t>
+          <t>密西西比灰鸢</t>
         </is>
       </c>
       <c r="F408" s="2" t="inlineStr">
@@ -18927,7 +18927,7 @@
       </c>
       <c r="E411" s="2" t="inlineStr">
         <is>
-          <t>和尚牡马</t>
+          <t>和尚鹦鹉</t>
         </is>
       </c>
       <c r="F411" s="2" t="inlineStr">
@@ -19111,7 +19111,7 @@
       </c>
       <c r="E415" s="2" t="inlineStr">
         <is>
-          <t>山翎禽</t>
+          <t>山翎鹑</t>
         </is>
       </c>
       <c r="F415" s="2" t="inlineStr">
@@ -19327,7 +19327,7 @@
       </c>
       <c r="E420" s="2" t="inlineStr">
         <is>
-          <t>南迪鹦鹉</t>
+          <t>黑头鹦哥</t>
         </is>
       </c>
       <c r="F420" s="2" t="inlineStr">
@@ -19459,7 +19459,7 @@
       </c>
       <c r="E423" s="2" t="inlineStr">
         <is>
-          <t>新西兰 达布奇克</t>
+          <t>新西兰䴙䴘</t>
         </is>
       </c>
       <c r="F423" s="2" t="inlineStr">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="E429" s="2" t="inlineStr">
         <is>
-          <t>吵闹的矿工</t>
+          <t>黑头矿鸟</t>
         </is>
       </c>
       <c r="F429" s="2" t="inlineStr">
@@ -19855,7 +19855,7 @@
       </c>
       <c r="E432" s="2" t="inlineStr">
         <is>
-          <t>山齿禽</t>
+          <t>山齿鹑</t>
         </is>
       </c>
       <c r="F432" s="2" t="inlineStr">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="E434" s="2" t="inlineStr">
         <is>
-          <t>北扑翅鴷</t>
+          <t>北扑翅䴕</t>
         </is>
       </c>
       <c r="F434" s="2" t="inlineStr">
@@ -20131,7 +20131,7 @@
       </c>
       <c r="E438" s="2" t="inlineStr">
         <is>
-          <t>小咯鸫</t>
+          <t>小嘲鸫</t>
         </is>
       </c>
       <c r="F438" s="2" t="inlineStr">
@@ -20227,7 +20227,7 @@
       </c>
       <c r="E440" s="2" t="inlineStr">
         <is>
-          <t>柬埔寨鬼鸮</t>
+          <t>棕榈鬼鸮</t>
         </is>
       </c>
       <c r="F440" s="2" t="inlineStr">
@@ -20875,7 +20875,7 @@
       </c>
       <c r="E454" s="2" t="inlineStr">
         <is>
-          <t>彩绘彩旗</t>
+          <t>丽彩鹀</t>
         </is>
       </c>
       <c r="F454" s="2" t="inlineStr">
@@ -20919,7 +20919,7 @@
       </c>
       <c r="E455" s="2" t="inlineStr">
         <is>
-          <t>彩绘白鸲</t>
+          <t>彩鸲莺</t>
         </is>
       </c>
       <c r="F455" s="2" t="inlineStr">
@@ -21043,7 +21043,7 @@
       </c>
       <c r="E458" s="2" t="inlineStr">
         <is>
-          <t>交紫嘴雀</t>
+          <t>鹦交嘴雀</t>
         </is>
       </c>
       <c r="F458" s="2" t="inlineStr">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="E462" s="2" t="inlineStr">
         <is>
-          <t>派斯奎特氏栗马</t>
+          <t>派斯奎特氏鹦鹉</t>
         </is>
       </c>
       <c r="F462" s="2" t="inlineStr">
@@ -21263,7 +21263,7 @@
       </c>
       <c r="E463" s="2" t="inlineStr">
         <is>
-          <t>菲诺贝普拉</t>
+          <t>亮丝鹟</t>
         </is>
       </c>
       <c r="F463" s="2" t="inlineStr">
@@ -21747,7 +21747,7 @@
       </c>
       <c r="E474" s="2" t="inlineStr">
         <is>
-          <t>领衔</t>
+          <t>领鹑</t>
         </is>
       </c>
       <c r="F474" s="2" t="inlineStr">
@@ -21883,7 +21883,7 @@
       </c>
       <c r="E477" s="2" t="inlineStr">
         <is>
-          <t>斯蒂芬妮公主的阿斯特拉皮亚</t>
+          <t>公主长尾天堂鸟</t>
         </is>
       </c>
       <c r="F477" s="2" t="inlineStr">
@@ -22007,7 +22007,7 @@
       </c>
       <c r="E480" s="2" t="inlineStr">
         <is>
-          <t>紫鸡</t>
+          <t>紫青水鸡</t>
         </is>
       </c>
       <c r="F480" s="2" t="inlineStr">
@@ -22195,7 +22195,7 @@
       </c>
       <c r="E484" s="2" t="inlineStr">
         <is>
-          <t>侏儒五子雀</t>
+          <t>侏䴓</t>
         </is>
       </c>
       <c r="F484" s="2" t="inlineStr">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="E485" s="2" t="inlineStr">
         <is>
-          <t>热毒症</t>
+          <t>灰额主红雀</t>
         </is>
       </c>
       <c r="F485" s="2" t="inlineStr">
@@ -22363,7 +22363,7 @@
       </c>
       <c r="E488" s="2" t="inlineStr">
         <is>
-          <t>彩虹吸蜜栗马</t>
+          <t>彩虹吸蜜鹦鹉</t>
         </is>
       </c>
       <c r="F488" s="2" t="inlineStr">
@@ -22843,7 +22843,7 @@
       </c>
       <c r="E498" s="2" t="inlineStr">
         <is>
-          <t>红嘴镰刀鸟</t>
+          <t>红嘴镰嘴鸟</t>
         </is>
       </c>
       <c r="F498" s="2" t="inlineStr">
@@ -23239,7 +23239,7 @@
       </c>
       <c r="E506" s="2" t="inlineStr">
         <is>
-          <t>红额栗马</t>
+          <t>红额鹦鹉</t>
         </is>
       </c>
       <c r="F506" s="2" t="inlineStr">
@@ -23387,7 +23387,7 @@
       </c>
       <c r="E509" s="2" t="inlineStr">
         <is>
-          <t>红头巴贝</t>
+          <t>红头拟啄木</t>
         </is>
       </c>
       <c r="F509" s="2" t="inlineStr">
@@ -23735,7 +23735,7 @@
       </c>
       <c r="E516" s="2" t="inlineStr">
         <is>
-          <t>黑喉红臀</t>
+          <t>黑喉红臀鹎</t>
         </is>
       </c>
       <c r="F516" s="2" t="inlineStr">
@@ -23891,7 +23891,7 @@
       </c>
       <c r="E519" s="2" t="inlineStr">
         <is>
-          <t>红紫牡马</t>
+          <t>红翅鹦鹉</t>
         </is>
       </c>
       <c r="F519" s="2" t="inlineStr">
@@ -24363,7 +24363,7 @@
       </c>
       <c r="E530" s="2" t="inlineStr">
         <is>
-          <t>红领绿褐马</t>
+          <t>红领绿鹦鹉</t>
         </is>
       </c>
       <c r="F530" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="E540" s="2" t="inlineStr">
         <is>
-          <t>红红虎鹭</t>
+          <t>栗虎斑鹭</t>
         </is>
       </c>
       <c r="F540" s="2" t="inlineStr">
@@ -24971,7 +24971,7 @@
       </c>
       <c r="E543" s="2" t="inlineStr">
         <is>
-          <t>棕黄蜂鸟</t>
+          <t>棕煌蜂鸟</t>
         </is>
       </c>
       <c r="F543" s="2" t="inlineStr">
@@ -25371,7 +25371,7 @@
       </c>
       <c r="E552" s="2" t="inlineStr">
         <is>
-          <t>沙丘克</t>
+          <t>沙丘鹤</t>
         </is>
       </c>
       <c r="F552" s="2" t="inlineStr">
@@ -25543,7 +25543,7 @@
       </c>
       <c r="E556" s="2" t="inlineStr">
         <is>
-          <t>稀树草原鹰</t>
+          <t>草原鸡𫛭</t>
         </is>
       </c>
       <c r="F556" s="2" t="inlineStr">
@@ -25683,7 +25683,7 @@
       </c>
       <c r="E559" s="2" t="inlineStr">
         <is>
-          <t>萨伊的菲比</t>
+          <t>塞氏菲比霸鹟</t>
         </is>
       </c>
       <c r="F559" s="2" t="inlineStr">
@@ -25731,7 +25731,7 @@
       </c>
       <c r="E560" s="2" t="inlineStr">
         <is>
-          <t>鳞斑猛兽</t>
+          <t>鳞斑鹑</t>
         </is>
       </c>
       <c r="F560" s="2" t="inlineStr">
@@ -25859,7 +25859,7 @@
       </c>
       <c r="E563" s="2" t="inlineStr">
         <is>
-          <t>绯红金刚棕马</t>
+          <t>绯红金刚鹦鹉</t>
         </is>
       </c>
       <c r="F563" s="2" t="inlineStr">
@@ -26255,7 +26255,7 @@
       </c>
       <c r="E572" s="2" t="inlineStr">
         <is>
-          <t>小迷你车</t>
+          <t>小山椒鸟</t>
         </is>
       </c>
       <c r="F572" s="2" t="inlineStr">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="E574" s="2" t="inlineStr">
         <is>
-          <t>滑嘴犀牛</t>
+          <t>滑嘴犀鹃</t>
         </is>
       </c>
       <c r="F574" s="2" t="inlineStr">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="E579" s="2" t="inlineStr">
         <is>
-          <t>歌带鵐</t>
+          <t>歌带鹀</t>
         </is>
       </c>
       <c r="F579" s="2" t="inlineStr">
@@ -26699,7 +26699,7 @@
       </c>
       <c r="E582" s="2" t="inlineStr">
         <is>
-          <t>鞍背鸦属</t>
+          <t>南岛鞍背鸦</t>
         </is>
       </c>
       <c r="F582" s="2" t="inlineStr">
@@ -26791,7 +26791,7 @@
       </c>
       <c r="E584" s="2" t="inlineStr">
         <is>
-          <t>南方鹤鹅</t>
+          <t>南方鹤鸵</t>
         </is>
       </c>
       <c r="F584" s="2" t="inlineStr">
@@ -27195,7 +27195,7 @@
       </c>
       <c r="E593" s="2" t="inlineStr">
         <is>
-          <t>一尘不染的椋鸟</t>
+          <t>纯色椋鸟</t>
         </is>
       </c>
       <c r="F593" s="2" t="inlineStr">
@@ -27363,7 +27363,7 @@
       </c>
       <c r="E597" s="2" t="inlineStr">
         <is>
-          <t>斑点海雀</t>
+          <t>斑蓬头䴕</t>
         </is>
       </c>
       <c r="F597" s="2" t="inlineStr">
@@ -27447,7 +27447,7 @@
       </c>
       <c r="E599" s="2" t="inlineStr">
         <is>
-          <t>斑点粗毛</t>
+          <t>点斑鸬鹚</t>
         </is>
       </c>
       <c r="F599" s="2" t="inlineStr">
@@ -27487,7 +27487,7 @@
       </c>
       <c r="E600" s="2" t="inlineStr">
         <is>
-          <t>斑驳鹀</t>
+          <t>斑唧鹀</t>
         </is>
       </c>
       <c r="F600" s="2" t="inlineStr">
@@ -27619,7 +27619,7 @@
       </c>
       <c r="E603" s="2" t="inlineStr">
         <is>
-          <t>腹灰棕棕</t>
+          <t>灰腹棕鹃</t>
         </is>
       </c>
       <c r="F603" s="2" t="inlineStr">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="E605" s="2" t="inlineStr">
         <is>
-          <t>斯里兰卡 蛙口鱼</t>
+          <t>斯里兰卡蟆口鸱</t>
         </is>
       </c>
       <c r="F605" s="2" t="inlineStr">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="E608" s="2" t="inlineStr">
         <is>
-          <t>僧吸蜜鸟</t>
+          <t>须吸蜜鸟</t>
         </is>
       </c>
       <c r="F608" s="2" t="inlineStr">
@@ -27943,7 +27943,7 @@
       </c>
       <c r="E610" s="2" t="inlineStr">
         <is>
-          <t>怪尾暴君</t>
+          <t>异尾霸鹟</t>
         </is>
       </c>
       <c r="F610" s="2" t="inlineStr">
@@ -28027,7 +28027,7 @@
       </c>
       <c r="E612" s="2" t="inlineStr">
         <is>
-          <t>葵花凤头栗马</t>
+          <t>葵花凤头鹦鹉</t>
         </is>
       </c>
       <c r="F612" s="2" t="inlineStr">
@@ -28075,7 +28075,7 @@
       </c>
       <c r="E613" s="2" t="inlineStr">
         <is>
-          <t>苏禄犀鸟</t>
+          <t>黑嘴斑犀鸟</t>
         </is>
       </c>
       <c r="F613" s="2" t="inlineStr">
@@ -28123,7 +28123,7 @@
       </c>
       <c r="E614" s="2" t="inlineStr">
         <is>
-          <t>太阳紫哥</t>
+          <t>太阳鹦哥</t>
         </is>
       </c>
       <c r="F614" s="2" t="inlineStr">
@@ -28563,7 +28563,7 @@
       </c>
       <c r="E624" s="2" t="inlineStr">
         <is>
-          <t>短翅鸊鷉</t>
+          <t>短翅䴙䴘</t>
         </is>
       </c>
       <c r="F624" s="2" t="inlineStr">
@@ -28815,7 +28815,7 @@
       </c>
       <c r="E630" s="2" t="inlineStr">
         <is>
-          <t>热带帕鲁拉</t>
+          <t>橄绿背森莺</t>
         </is>
       </c>
       <c r="F630" s="2" t="inlineStr">
@@ -28859,7 +28859,7 @@
       </c>
       <c r="E631" s="2" t="inlineStr">
         <is>
-          <t>热带皇家鹟</t>
+          <t>亚马逊王霸鹟</t>
         </is>
       </c>
       <c r="F631" s="2" t="inlineStr">
@@ -28983,7 +28983,7 @@
       </c>
       <c r="E634" s="2" t="inlineStr">
         <is>
-          <t>簇羽海紫</t>
+          <t>簇羽海鹦</t>
         </is>
       </c>
       <c r="F634" s="2" t="inlineStr">
@@ -29299,7 +29299,7 @@
       </c>
       <c r="E641" s="2" t="inlineStr">
         <is>
-          <t>群青粗喙鸟</t>
+          <t>深蓝彩鹀</t>
         </is>
       </c>
       <c r="F641" s="2" t="inlineStr">
@@ -29387,7 +29387,7 @@
       </c>
       <c r="E643" s="2" t="inlineStr">
         <is>
-          <t>可变蛎鹬</t>
+          <t>新西兰蛎鹬</t>
         </is>
       </c>
       <c r="F643" s="2" t="inlineStr">
@@ -29427,7 +29427,7 @@
       </c>
       <c r="E644" s="2" t="inlineStr">
         <is>
-          <t>可变播种机</t>
+          <t>杂色食籽雀</t>
         </is>
       </c>
       <c r="F644" s="2" t="inlineStr">
@@ -29551,7 +29551,7 @@
       </c>
       <c r="E647" s="2" t="inlineStr">
         <is>
-          <t>韦尔丁</t>
+          <t>黄头金雀</t>
         </is>
       </c>
       <c r="F647" s="2" t="inlineStr">
@@ -29639,7 +29639,7 @@
       </c>
       <c r="E649" s="2" t="inlineStr">
         <is>
-          <t>朱鹟</t>
+          <t>朱红霸鹟</t>
         </is>
       </c>
       <c r="F649" s="2" t="inlineStr">
@@ -29683,7 +29683,7 @@
       </c>
       <c r="E650" s="2" t="inlineStr">
         <is>
-          <t>紫金葫芦</t>
+          <t>紫金鹃</t>
         </is>
       </c>
       <c r="F650" s="2" t="inlineStr">
@@ -30359,7 +30359,7 @@
       </c>
       <c r="E665" s="2" t="inlineStr">
         <is>
-          <t>胡须树迅捷</t>
+          <t>小须凤头雨燕</t>
         </is>
       </c>
       <c r="F665" s="2" t="inlineStr">
@@ -30703,7 +30703,7 @@
       </c>
       <c r="E672" s="2" t="inlineStr">
         <is>
-          <t>白眉山雀</t>
+          <t>秘鲁白眉针尾雀</t>
         </is>
       </c>
       <c r="F672" s="2" t="inlineStr">
@@ -31259,7 +31259,7 @@
       </c>
       <c r="E683" s="2" t="inlineStr">
         <is>
-          <t>白额浅翅</t>
+          <t>白额棕翅鸠</t>
         </is>
       </c>
       <c r="F683" s="2" t="inlineStr">
@@ -31599,7 +31599,7 @@
       </c>
       <c r="E691" s="2" t="inlineStr">
         <is>
-          <t>美洲沙锥</t>
+          <t>威氏鹬</t>
         </is>
       </c>
       <c r="F691" s="2" t="inlineStr">
@@ -32071,7 +32071,7 @@
       </c>
       <c r="E701" s="2" t="inlineStr">
         <is>
-          <t>黄胸大𱉼莺</t>
+          <t>黄胸巨鵖莺</t>
         </is>
       </c>
       <c r="F701" s="2" t="inlineStr">
@@ -33195,7 +33195,7 @@
       </c>
       <c r="E729" s="2" t="inlineStr">
         <is>
-          <t>红尾慧星蜂鸟</t>
+          <t>红尾彗星蜂鸟</t>
         </is>
       </c>
       <c r="F729" s="2" t="n"/>
@@ -33675,7 +33675,7 @@
       </c>
       <c r="E742" s="2" t="inlineStr">
         <is>
-          <t>燕尾刀翅翅鸟</t>
+          <t>燕尾刀翅蜂鸟</t>
         </is>
       </c>
       <c r="F742" s="2" t="n"/>
@@ -33747,7 +33747,7 @@
       </c>
       <c r="E744" s="2" t="inlineStr">
         <is>
-          <t>紫刀翅翅鸟</t>
+          <t>紫刀翅蜂鸟</t>
         </is>
       </c>
       <c r="F744" s="2" t="n"/>

</xml_diff>